<commit_message>
Rename the method to hemodynamic attenuation (the score stays the collateral value) in figures, paper, notebooks and workbook; Optimal Brain Damage cited as 1989; Michel-style and Voita-style rows, noting the published methods are run inside our training; Figure 2 caption matches the new panels
</commit_message>
<xml_diff>
--- a/notebooks/hmha_by_hand.xlsx
+++ b/notebooks/hmha_by_hand.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mason\CODE2026\HMHA\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A92E345-EA72-46DE-8DB3-848B80238D74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BAED533-0126-45D3-9ADF-BF97AA61F44D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="480" yWindow="1230" windowWidth="27180" windowHeight="17610" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="499">
   <si>
-    <t>The collateral rule by hand: the whole project on a tiny task</t>
+    <t>Hemodynamic attenuation by hand: the whole project on a tiny task</t>
   </si>
   <si>
     <t>Each sheet is one step. Work through them in order: 1 Task, 2 One head, 3 Two heads, 4 Why R heads,</t>

</xml_diff>